<commit_message>
added uORFs to TableS5 for now
</commit_message>
<xml_diff>
--- a/Supplemental Files/Table S5.xlsx
+++ b/Supplemental Files/Table S5.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Šimon Pavlů\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B949B559-6B1F-4555-9E5A-F731BD4A2B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976B09F8-DE03-49EA-8C2C-3C28200D5C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F43FCF7E-9F21-478D-94EF-A6D81F31AE0B}"/>
   </bookViews>
   <sheets>
-    <sheet name="TableS5A" sheetId="5" r:id="rId1"/>
-    <sheet name="TableS5B" sheetId="6" r:id="rId2"/>
-    <sheet name="TableS5C" sheetId="1" r:id="rId3"/>
+    <sheet name="uORFs" sheetId="7" r:id="rId1"/>
+    <sheet name="TableS5A" sheetId="5" r:id="rId2"/>
+    <sheet name="TableS5B" sheetId="6" r:id="rId3"/>
+    <sheet name="TableS5C" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">TableS5B!$A$3:$L$1559</definedName>
+    <definedName name="ExternalData_1" localSheetId="2" hidden="1">TableS5B!$A$3:$L$1559</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15473" uniqueCount="1907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15881" uniqueCount="2308">
   <si>
     <t># -----------------</t>
   </si>
@@ -5773,6 +5774,1209 @@
   </si>
   <si>
     <t>ABC transporter G family member</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0004310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0005830</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0012730</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0013180</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0015110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0018170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0019100</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0019340</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0019730</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0030010</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0044840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0046580</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0049980</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0051380</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0052800</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0053250</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0055840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0058270</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0059070</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0059910</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0060380</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0065840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0066150</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0067010</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0067260</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0068060</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0068750</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0069010</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0069250</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0072760</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0072880</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0073570</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0073900</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0077310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0079120</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0086540</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0088700</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.1HG0090050</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0096370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0099800</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0102870</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0107470</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0110560</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0111000</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0111570</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0113290</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0114840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0119970</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0124680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0128960</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0132990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0133550</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0133890</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0143300</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0146160</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0146430</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0150440</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0152470</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0153420</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0162930</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0164700</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0165180</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0166910</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0170290</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0171960</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0173230</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0173400</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0174620</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0174680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0174980</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0176030</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0179320</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0180110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0181540</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0182020</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0183370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0184460</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0185210</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0185770</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0186340</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0190260</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0191120</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0193170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0195110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0200780</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0200990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0203380</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0204030</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0205510</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0206700</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0209210</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0214820</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.2HG0215190</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0222830</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0223370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0224410</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0228120</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0228170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0230380</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0232310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0233790</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0234500</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0236780</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0243960</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0244000</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0245400</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0246180</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0248290</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0249020</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0249160</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0249930</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0250060</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0252000</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0254550</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0254600</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0255050</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0258000</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0258640</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0264400</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0266810</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0267140</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0270050</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0271580</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0275260</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0276890</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0278140</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0278540</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0279110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0279530</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0280980</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0283080</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0283450</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0284870</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0285860</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0286190</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0290670</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0290960</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0292470</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0296100</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0296310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0297270</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0298320</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0298800</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0301040</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0302730</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0303130</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0303560</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0305280</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0308630</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0310930</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0311480</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0316900</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0318260</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0318390</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0319370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0323770</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0329000</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0330450</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.3HG0330950</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0333550</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0333630</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0333850</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0334370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0334980</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0335230</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0338590</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0338770</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0341500</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0344270</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0347400</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0347680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0348550</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0348970</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0351440</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0354250</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0355210</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0355410</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0356550</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0358480</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0362850</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0362920</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0369610</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0376510</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0379920</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0380710</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0383230</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0383400</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0383790</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0389620</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0390200</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0391110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0391260</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0391910</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0394680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0394990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0395220</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0396540</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0399110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0402070</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0404190</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0405890</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0408090</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0408100</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0408620</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0409170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0410700</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0411110</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0411520</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0412030</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0412770</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0412790</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0413050</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0413890</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0414140</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0414940</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0414960</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0416570</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.4HG0418520</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0419880</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0420170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0420370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0420380</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0423810</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0423820</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0428330</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0428850</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0432640</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0436650</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0438160</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0438310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0439250</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0439640</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0440150</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0440800</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0441840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0442860</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0443020</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0454720</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0460560</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0462760</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0463700</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0466060</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0466930</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0468700</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0468930</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0470480</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0471520</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0475180</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0477590</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0479750</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0480800</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0482370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0482640</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0483030</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0484020</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0484230</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0489020</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0489840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0491030</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0491580</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0492170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0494170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0498130</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0498270</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0498710</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0498810</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0498890</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0499030</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0502300</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0502680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0503060</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0504220</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0504980</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0506720</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0506790</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0509680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0509970</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0510640</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0512150</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0512230</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0512370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0512710</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0513310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0516400</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0516590</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0517240</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0517490</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0523330</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0523860</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0524300</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0529780</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0530740</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0530780</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0531390</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0533230</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.5HG0534990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0546530</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0548250</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0554970</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0557160</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0557190</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0566220</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0573070</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0573080</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0573200</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0573300</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0573510</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0574430</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0574950</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0585610</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0585990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0589180</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0589470</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0589640</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0590990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0591450</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0593300</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0593860</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0594260</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0597350</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0601990</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0603120</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0604470</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0605460</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0605810</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0607410</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0608170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0611210</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0612510</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0614460</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0614470</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0616560</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0617920</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0620390</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0620650</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0621790</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0623790</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0624390</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0625130</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0627070</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0627480</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0627540</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0632680</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.6HG0633430</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0638370</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0639360</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0639890</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0640390</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0644570</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0653180</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0654310</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0656840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0656930</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0657100</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0657870</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0660620</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0661420</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0662630</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0665730</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0666290</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0671350</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0673000</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0677380</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0677440</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0678530</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0680520</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0682660</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0683560</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0689530</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0692590</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0696190</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0697980</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0700220</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0702610</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0709070</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0709880</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0711300</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0711580</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0713020</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0714440</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0714570</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0719170</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0719440</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0723120</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0723280</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0724740</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0725050</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0726750</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0728390</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0731430</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0732860</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0740760</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0745800</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0746840</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0747100</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0748160</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0750280</t>
+  </si>
+  <si>
+    <t>HORVU.MOREX.r3.7HG0750360</t>
+  </si>
+  <si>
+    <t>Gene ID</t>
+  </si>
+  <si>
+    <t>uORF</t>
+  </si>
+  <si>
+    <t>TableS5X. Genes with promoter shift and potential uORFs located within the region between two shifting TSSs.</t>
   </si>
 </sst>
 </file>
@@ -6267,6 +7471,3272 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3627361A-395D-4621-8140-640E9E873244}">
+  <dimension ref="A1:B408"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>2305</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2306</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>1907</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1908</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>1909</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>1910</v>
+      </c>
+      <c r="B7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>1911</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>1913</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>1914</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>1915</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>1916</v>
+      </c>
+      <c r="B13">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>1917</v>
+      </c>
+      <c r="B14">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>1918</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1919</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1920</v>
+      </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>1921</v>
+      </c>
+      <c r="B18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>1922</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>1923</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>1924</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>1925</v>
+      </c>
+      <c r="B22">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>1926</v>
+      </c>
+      <c r="B23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>1927</v>
+      </c>
+      <c r="B24">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>1928</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>1929</v>
+      </c>
+      <c r="B26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>1930</v>
+      </c>
+      <c r="B27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>1931</v>
+      </c>
+      <c r="B28">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>1932</v>
+      </c>
+      <c r="B29">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>1933</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>1934</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>1935</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>1936</v>
+      </c>
+      <c r="B33">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>1937</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>1938</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>1940</v>
+      </c>
+      <c r="B37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>1941</v>
+      </c>
+      <c r="B38">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>1942</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>1943</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>1944</v>
+      </c>
+      <c r="B41">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B42">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>1946</v>
+      </c>
+      <c r="B43">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>1947</v>
+      </c>
+      <c r="B44">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>1948</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>1949</v>
+      </c>
+      <c r="B46">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>1950</v>
+      </c>
+      <c r="B47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>1951</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>1953</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>46</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>1954</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B53">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>1956</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>1957</v>
+      </c>
+      <c r="B55">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>1958</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>1959</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>1960</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>1961</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>1962</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>1964</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>1965</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>1966</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>1967</v>
+      </c>
+      <c r="B65">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>1968</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>1970</v>
+      </c>
+      <c r="B68">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>1971</v>
+      </c>
+      <c r="B69">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>1972</v>
+      </c>
+      <c r="B70">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>1973</v>
+      </c>
+      <c r="B71">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>1974</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>1975</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>1976</v>
+      </c>
+      <c r="B74">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>1977</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>1978</v>
+      </c>
+      <c r="B76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>1979</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>1980</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>1981</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>1982</v>
+      </c>
+      <c r="B80">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B81">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>1984</v>
+      </c>
+      <c r="B82">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>1985</v>
+      </c>
+      <c r="B83">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>1986</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B85">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>1988</v>
+      </c>
+      <c r="B86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>1989</v>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>1990</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>74</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>1991</v>
+      </c>
+      <c r="B90">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>1992</v>
+      </c>
+      <c r="B91">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>1993</v>
+      </c>
+      <c r="B92">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>1994</v>
+      </c>
+      <c r="B93">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>1995</v>
+      </c>
+      <c r="B94">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>1996</v>
+      </c>
+      <c r="B95">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>1997</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>1998</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>1999</v>
+      </c>
+      <c r="B98">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>2000</v>
+      </c>
+      <c r="B99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>2001</v>
+      </c>
+      <c r="B100">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>2002</v>
+      </c>
+      <c r="B101">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>2003</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>2004</v>
+      </c>
+      <c r="B103">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>2006</v>
+      </c>
+      <c r="B105">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>2007</v>
+      </c>
+      <c r="B106">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B107">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>2009</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>2010</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>2011</v>
+      </c>
+      <c r="B110">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>2013</v>
+      </c>
+      <c r="B112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>2014</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>2015</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>2017</v>
+      </c>
+      <c r="B116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>2018</v>
+      </c>
+      <c r="B117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>2019</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>2020</v>
+      </c>
+      <c r="B119">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>2021</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>2022</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>2023</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B123">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>2025</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>2026</v>
+      </c>
+      <c r="B125">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>2027</v>
+      </c>
+      <c r="B126">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B127">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>2029</v>
+      </c>
+      <c r="B128">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>2030</v>
+      </c>
+      <c r="B129">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B130">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>2032</v>
+      </c>
+      <c r="B131">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>2033</v>
+      </c>
+      <c r="B132">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B133">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>2035</v>
+      </c>
+      <c r="B134">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>2036</v>
+      </c>
+      <c r="B135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B136">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>2038</v>
+      </c>
+      <c r="B137">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>2039</v>
+      </c>
+      <c r="B138">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>2040</v>
+      </c>
+      <c r="B139">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>2041</v>
+      </c>
+      <c r="B140">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>2042</v>
+      </c>
+      <c r="B141">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>2043</v>
+      </c>
+      <c r="B142">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>2044</v>
+      </c>
+      <c r="B143">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>105</v>
+      </c>
+      <c r="B144">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B145">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>2046</v>
+      </c>
+      <c r="B146">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>107</v>
+      </c>
+      <c r="B147">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>2047</v>
+      </c>
+      <c r="B148">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>2048</v>
+      </c>
+      <c r="B149">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B150">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>2050</v>
+      </c>
+      <c r="B151">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>2051</v>
+      </c>
+      <c r="B152">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B153">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>2053</v>
+      </c>
+      <c r="B154">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>2054</v>
+      </c>
+      <c r="B155">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B156">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>2056</v>
+      </c>
+      <c r="B157">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>2057</v>
+      </c>
+      <c r="B158">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>2058</v>
+      </c>
+      <c r="B159">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>2059</v>
+      </c>
+      <c r="B160">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>2060</v>
+      </c>
+      <c r="B161">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>2061</v>
+      </c>
+      <c r="B162">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>2062</v>
+      </c>
+      <c r="B163">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>2063</v>
+      </c>
+      <c r="B164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>2064</v>
+      </c>
+      <c r="B165">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>2065</v>
+      </c>
+      <c r="B166">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>2066</v>
+      </c>
+      <c r="B167">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>2067</v>
+      </c>
+      <c r="B168">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>2068</v>
+      </c>
+      <c r="B169">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>2069</v>
+      </c>
+      <c r="B170">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B171">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>2071</v>
+      </c>
+      <c r="B172">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>2072</v>
+      </c>
+      <c r="B173">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>2073</v>
+      </c>
+      <c r="B174">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>2074</v>
+      </c>
+      <c r="B175">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B176">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>2076</v>
+      </c>
+      <c r="B177">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>2077</v>
+      </c>
+      <c r="B178">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>2078</v>
+      </c>
+      <c r="B179">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>2079</v>
+      </c>
+      <c r="B180">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B181">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>2081</v>
+      </c>
+      <c r="B182">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>2082</v>
+      </c>
+      <c r="B183">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>2083</v>
+      </c>
+      <c r="B184">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>2084</v>
+      </c>
+      <c r="B185">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B186">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>2086</v>
+      </c>
+      <c r="B187">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>2087</v>
+      </c>
+      <c r="B188">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>2088</v>
+      </c>
+      <c r="B189">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>2089</v>
+      </c>
+      <c r="B190">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>2090</v>
+      </c>
+      <c r="B191">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>2091</v>
+      </c>
+      <c r="B192">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>2092</v>
+      </c>
+      <c r="B193">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>2093</v>
+      </c>
+      <c r="B194">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>2094</v>
+      </c>
+      <c r="B195">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>127</v>
+      </c>
+      <c r="B196">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>2095</v>
+      </c>
+      <c r="B197">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>2096</v>
+      </c>
+      <c r="B198">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>2097</v>
+      </c>
+      <c r="B199">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B200">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>2099</v>
+      </c>
+      <c r="B201">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>2100</v>
+      </c>
+      <c r="B202">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>2101</v>
+      </c>
+      <c r="B203">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>2102</v>
+      </c>
+      <c r="B204">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>2103</v>
+      </c>
+      <c r="B205">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>2104</v>
+      </c>
+      <c r="B206">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>2105</v>
+      </c>
+      <c r="B207">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>2106</v>
+      </c>
+      <c r="B208">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>2107</v>
+      </c>
+      <c r="B209">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>2108</v>
+      </c>
+      <c r="B210">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>2109</v>
+      </c>
+      <c r="B211">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>2110</v>
+      </c>
+      <c r="B212">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>2111</v>
+      </c>
+      <c r="B213">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>2112</v>
+      </c>
+      <c r="B214">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>2113</v>
+      </c>
+      <c r="B215">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>2114</v>
+      </c>
+      <c r="B216">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>2115</v>
+      </c>
+      <c r="B217">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>2116</v>
+      </c>
+      <c r="B218">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>2117</v>
+      </c>
+      <c r="B219">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B220">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>2119</v>
+      </c>
+      <c r="B221">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>2120</v>
+      </c>
+      <c r="B222">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>2121</v>
+      </c>
+      <c r="B223">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>2122</v>
+      </c>
+      <c r="B224">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>2123</v>
+      </c>
+      <c r="B225">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>2124</v>
+      </c>
+      <c r="B226">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>2125</v>
+      </c>
+      <c r="B227">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B228">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>2127</v>
+      </c>
+      <c r="B229">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>2128</v>
+      </c>
+      <c r="B230">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>2129</v>
+      </c>
+      <c r="B231">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>2130</v>
+      </c>
+      <c r="B232">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>2131</v>
+      </c>
+      <c r="B233">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>2132</v>
+      </c>
+      <c r="B234">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>2133</v>
+      </c>
+      <c r="B235">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>2134</v>
+      </c>
+      <c r="B236">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>2135</v>
+      </c>
+      <c r="B237">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>2136</v>
+      </c>
+      <c r="B238">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>2137</v>
+      </c>
+      <c r="B239">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>2138</v>
+      </c>
+      <c r="B240">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>2139</v>
+      </c>
+      <c r="B241">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>2140</v>
+      </c>
+      <c r="B242">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A243" t="s">
+        <v>2141</v>
+      </c>
+      <c r="B243">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A244" t="s">
+        <v>2142</v>
+      </c>
+      <c r="B244">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A245" t="s">
+        <v>2143</v>
+      </c>
+      <c r="B245">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A246" t="s">
+        <v>2144</v>
+      </c>
+      <c r="B246">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A247" t="s">
+        <v>2145</v>
+      </c>
+      <c r="B247">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A248" t="s">
+        <v>2146</v>
+      </c>
+      <c r="B248">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A249" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B249">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A250" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B250">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A251" t="s">
+        <v>2149</v>
+      </c>
+      <c r="B251">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A252" t="s">
+        <v>2150</v>
+      </c>
+      <c r="B252">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A253" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B253">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A254" t="s">
+        <v>2152</v>
+      </c>
+      <c r="B254">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A255" t="s">
+        <v>2153</v>
+      </c>
+      <c r="B255">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A256" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B256">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A257" t="s">
+        <v>2155</v>
+      </c>
+      <c r="B257">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A258" t="s">
+        <v>2156</v>
+      </c>
+      <c r="B258">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A259" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B259">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A260" t="s">
+        <v>2158</v>
+      </c>
+      <c r="B260">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A261" t="s">
+        <v>2159</v>
+      </c>
+      <c r="B261">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A262" t="s">
+        <v>2160</v>
+      </c>
+      <c r="B262">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A263" t="s">
+        <v>2161</v>
+      </c>
+      <c r="B263">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A264" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B264">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A265" t="s">
+        <v>157</v>
+      </c>
+      <c r="B265">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A266" t="s">
+        <v>2163</v>
+      </c>
+      <c r="B266">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A267" t="s">
+        <v>2164</v>
+      </c>
+      <c r="B267">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A268" t="s">
+        <v>2165</v>
+      </c>
+      <c r="B268">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A269" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B269">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A270" t="s">
+        <v>2167</v>
+      </c>
+      <c r="B270">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A271" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B271">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A272" t="s">
+        <v>2169</v>
+      </c>
+      <c r="B272">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A273" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B273">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A274" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B274">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A275" t="s">
+        <v>2172</v>
+      </c>
+      <c r="B275">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A276" t="s">
+        <v>2173</v>
+      </c>
+      <c r="B276">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A277" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B277">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A278" t="s">
+        <v>2175</v>
+      </c>
+      <c r="B278">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A279" t="s">
+        <v>2176</v>
+      </c>
+      <c r="B279">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A280" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B280">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A281" t="s">
+        <v>2178</v>
+      </c>
+      <c r="B281">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A282" t="s">
+        <v>2179</v>
+      </c>
+      <c r="B282">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A283" t="s">
+        <v>2180</v>
+      </c>
+      <c r="B283">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A284" t="s">
+        <v>2181</v>
+      </c>
+      <c r="B284">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A285" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B285">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A286" t="s">
+        <v>2183</v>
+      </c>
+      <c r="B286">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A287" t="s">
+        <v>2184</v>
+      </c>
+      <c r="B287">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>2185</v>
+      </c>
+      <c r="B288">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A289" t="s">
+        <v>2186</v>
+      </c>
+      <c r="B289">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A290" t="s">
+        <v>2187</v>
+      </c>
+      <c r="B290">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A291" t="s">
+        <v>2188</v>
+      </c>
+      <c r="B291">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A292" t="s">
+        <v>2189</v>
+      </c>
+      <c r="B292">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A293" t="s">
+        <v>2190</v>
+      </c>
+      <c r="B293">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A294" t="s">
+        <v>2191</v>
+      </c>
+      <c r="B294">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A295" t="s">
+        <v>2192</v>
+      </c>
+      <c r="B295">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A296" t="s">
+        <v>2193</v>
+      </c>
+      <c r="B296">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A297" t="s">
+        <v>2194</v>
+      </c>
+      <c r="B297">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A298" t="s">
+        <v>2195</v>
+      </c>
+      <c r="B298">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A299" t="s">
+        <v>2196</v>
+      </c>
+      <c r="B299">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A300" t="s">
+        <v>2197</v>
+      </c>
+      <c r="B300">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A301" t="s">
+        <v>2198</v>
+      </c>
+      <c r="B301">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A302" t="s">
+        <v>2199</v>
+      </c>
+      <c r="B302">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A303" t="s">
+        <v>2200</v>
+      </c>
+      <c r="B303">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A304" t="s">
+        <v>2201</v>
+      </c>
+      <c r="B304">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A305" t="s">
+        <v>2202</v>
+      </c>
+      <c r="B305">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A306" t="s">
+        <v>2203</v>
+      </c>
+      <c r="B306">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A307" t="s">
+        <v>2204</v>
+      </c>
+      <c r="B307">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A308" t="s">
+        <v>2205</v>
+      </c>
+      <c r="B308">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A309" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B309">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A310" t="s">
+        <v>2207</v>
+      </c>
+      <c r="B310">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A311" t="s">
+        <v>2208</v>
+      </c>
+      <c r="B311">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A312" t="s">
+        <v>2209</v>
+      </c>
+      <c r="B312">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A313" t="s">
+        <v>2210</v>
+      </c>
+      <c r="B313">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A314" t="s">
+        <v>2211</v>
+      </c>
+      <c r="B314">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A315" t="s">
+        <v>2212</v>
+      </c>
+      <c r="B315">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A316" t="s">
+        <v>2213</v>
+      </c>
+      <c r="B316">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A317" t="s">
+        <v>2214</v>
+      </c>
+      <c r="B317">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A318" t="s">
+        <v>2215</v>
+      </c>
+      <c r="B318">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A319" t="s">
+        <v>2216</v>
+      </c>
+      <c r="B319">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A320" t="s">
+        <v>2217</v>
+      </c>
+      <c r="B320">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A321" t="s">
+        <v>2218</v>
+      </c>
+      <c r="B321">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A322" t="s">
+        <v>2219</v>
+      </c>
+      <c r="B322">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A323" t="s">
+        <v>2220</v>
+      </c>
+      <c r="B323">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A324" t="s">
+        <v>2221</v>
+      </c>
+      <c r="B324">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A325" t="s">
+        <v>2222</v>
+      </c>
+      <c r="B325">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A326" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B326">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A327" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B327">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A328" t="s">
+        <v>2225</v>
+      </c>
+      <c r="B328">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A329" t="s">
+        <v>2226</v>
+      </c>
+      <c r="B329">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A330" t="s">
+        <v>2227</v>
+      </c>
+      <c r="B330">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A331" t="s">
+        <v>2228</v>
+      </c>
+      <c r="B331">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A332" t="s">
+        <v>2229</v>
+      </c>
+      <c r="B332">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A333" t="s">
+        <v>2230</v>
+      </c>
+      <c r="B333">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A334" t="s">
+        <v>2231</v>
+      </c>
+      <c r="B334">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A335" t="s">
+        <v>2232</v>
+      </c>
+      <c r="B335">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A336" t="s">
+        <v>2233</v>
+      </c>
+      <c r="B336">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A337" t="s">
+        <v>2234</v>
+      </c>
+      <c r="B337">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A338" t="s">
+        <v>2235</v>
+      </c>
+      <c r="B338">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A339" t="s">
+        <v>2236</v>
+      </c>
+      <c r="B339">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A340" t="s">
+        <v>2237</v>
+      </c>
+      <c r="B340">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A341" t="s">
+        <v>2238</v>
+      </c>
+      <c r="B341">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A342" t="s">
+        <v>2239</v>
+      </c>
+      <c r="B342">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A343" t="s">
+        <v>2240</v>
+      </c>
+      <c r="B343">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A344" t="s">
+        <v>2241</v>
+      </c>
+      <c r="B344">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A345" t="s">
+        <v>2242</v>
+      </c>
+      <c r="B345">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A346" t="s">
+        <v>2243</v>
+      </c>
+      <c r="B346">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A347" t="s">
+        <v>2244</v>
+      </c>
+      <c r="B347">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A348" t="s">
+        <v>2245</v>
+      </c>
+      <c r="B348">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A349" t="s">
+        <v>2246</v>
+      </c>
+      <c r="B349">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A350" t="s">
+        <v>2247</v>
+      </c>
+      <c r="B350">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A351" t="s">
+        <v>2248</v>
+      </c>
+      <c r="B351">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A352" t="s">
+        <v>2249</v>
+      </c>
+      <c r="B352">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A353" t="s">
+        <v>2250</v>
+      </c>
+      <c r="B353">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A354" t="s">
+        <v>2251</v>
+      </c>
+      <c r="B354">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A355" t="s">
+        <v>2252</v>
+      </c>
+      <c r="B355">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A356" t="s">
+        <v>2253</v>
+      </c>
+      <c r="B356">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A357" t="s">
+        <v>2254</v>
+      </c>
+      <c r="B357">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A358" t="s">
+        <v>2255</v>
+      </c>
+      <c r="B358">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A359" t="s">
+        <v>2256</v>
+      </c>
+      <c r="B359">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A360" t="s">
+        <v>2257</v>
+      </c>
+      <c r="B360">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A361" t="s">
+        <v>2258</v>
+      </c>
+      <c r="B361">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A362" t="s">
+        <v>2259</v>
+      </c>
+      <c r="B362">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A363" t="s">
+        <v>2260</v>
+      </c>
+      <c r="B363">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A364" t="s">
+        <v>2261</v>
+      </c>
+      <c r="B364">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A365" t="s">
+        <v>2262</v>
+      </c>
+      <c r="B365">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A366" t="s">
+        <v>2263</v>
+      </c>
+      <c r="B366">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A367" t="s">
+        <v>2264</v>
+      </c>
+      <c r="B367">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A368" t="s">
+        <v>2265</v>
+      </c>
+      <c r="B368">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A369" t="s">
+        <v>2266</v>
+      </c>
+      <c r="B369">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A370" t="s">
+        <v>2267</v>
+      </c>
+      <c r="B370">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A371" t="s">
+        <v>2268</v>
+      </c>
+      <c r="B371">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A372" t="s">
+        <v>2269</v>
+      </c>
+      <c r="B372">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A373" t="s">
+        <v>2270</v>
+      </c>
+      <c r="B373">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A374" t="s">
+        <v>2271</v>
+      </c>
+      <c r="B374">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A375" t="s">
+        <v>2272</v>
+      </c>
+      <c r="B375">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A376" t="s">
+        <v>2273</v>
+      </c>
+      <c r="B376">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A377" t="s">
+        <v>2274</v>
+      </c>
+      <c r="B377">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A378" t="s">
+        <v>2275</v>
+      </c>
+      <c r="B378">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A379" t="s">
+        <v>2276</v>
+      </c>
+      <c r="B379">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A380" t="s">
+        <v>2277</v>
+      </c>
+      <c r="B380">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A381" t="s">
+        <v>2278</v>
+      </c>
+      <c r="B381">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A382" t="s">
+        <v>2279</v>
+      </c>
+      <c r="B382">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A383" t="s">
+        <v>2280</v>
+      </c>
+      <c r="B383">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A384" t="s">
+        <v>241</v>
+      </c>
+      <c r="B384">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A385" t="s">
+        <v>2281</v>
+      </c>
+      <c r="B385">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A386" t="s">
+        <v>2282</v>
+      </c>
+      <c r="B386">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A387" t="s">
+        <v>2283</v>
+      </c>
+      <c r="B387">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A388" t="s">
+        <v>2284</v>
+      </c>
+      <c r="B388">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A389" t="s">
+        <v>2285</v>
+      </c>
+      <c r="B389">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A390" t="s">
+        <v>2286</v>
+      </c>
+      <c r="B390">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A391" t="s">
+        <v>2287</v>
+      </c>
+      <c r="B391">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A392" t="s">
+        <v>2288</v>
+      </c>
+      <c r="B392">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A393" t="s">
+        <v>2289</v>
+      </c>
+      <c r="B393">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A394" t="s">
+        <v>2290</v>
+      </c>
+      <c r="B394">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A395" t="s">
+        <v>2291</v>
+      </c>
+      <c r="B395">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A396" t="s">
+        <v>2292</v>
+      </c>
+      <c r="B396">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A397" t="s">
+        <v>2293</v>
+      </c>
+      <c r="B397">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A398" t="s">
+        <v>2294</v>
+      </c>
+      <c r="B398">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A399" t="s">
+        <v>2295</v>
+      </c>
+      <c r="B399">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A400" t="s">
+        <v>2296</v>
+      </c>
+      <c r="B400">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A401" t="s">
+        <v>2297</v>
+      </c>
+      <c r="B401">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A402" t="s">
+        <v>2298</v>
+      </c>
+      <c r="B402">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A403" t="s">
+        <v>2299</v>
+      </c>
+      <c r="B403">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A404" t="s">
+        <v>2300</v>
+      </c>
+      <c r="B404">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A405" t="s">
+        <v>2301</v>
+      </c>
+      <c r="B405">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A406" t="s">
+        <v>2302</v>
+      </c>
+      <c r="B406">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A407" t="s">
+        <v>2303</v>
+      </c>
+      <c r="B407">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A408" t="s">
+        <v>2304</v>
+      </c>
+      <c r="B408">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{710AC752-BA6D-4333-A4EB-D5CE54B48E9A}">
   <dimension ref="A1:K270"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -15678,7 +20148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7865610B-85E1-495C-A84C-699D7D0DFF15}">
   <dimension ref="A1:L1559"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -74879,7 +79349,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6A37F7F-7B8A-45B2-8023-BDD9EE2375D6}">
   <dimension ref="A1:M178"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>